<commit_message>
Updated and added more info to Ex2B
</commit_message>
<xml_diff>
--- a/week-01/Ex2B_data_roundup.xlsx
+++ b/week-01/Ex2B_data_roundup.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marenzasantarin\OneDrive - Year Up- BOS\Documents\DataAnalytics\week-01\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA4BAAE4-EE80-4321-8ACE-2F5DDE959583}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7488AB58-A616-4D68-A8BA-D1DEC6A76D22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{BB5919B5-10CD-4854-8E8E-8FD2EB376CE8}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BB5919B5-10CD-4854-8E8E-8FD2EB376CE8}"/>
   </bookViews>
   <sheets>
     <sheet name="Ex2B_Personal_Data_Roundup" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="25">
   <si>
     <t>Downloadable?</t>
   </si>
@@ -62,39 +62,15 @@
     <t>Bank account</t>
   </si>
   <si>
-    <t>Financial / purchases / Services</t>
-  </si>
-  <si>
     <t>Months to years</t>
   </si>
   <si>
     <t>Yes</t>
   </si>
   <si>
-    <t>Log in &gt; Statements or transaction history &gt; Download or Export</t>
-  </si>
-  <si>
-    <t>.pdf or .csv</t>
-  </si>
-  <si>
     <t>Some banks limit export range by month or statement period.</t>
   </si>
   <si>
-    <t>Gmail</t>
-  </si>
-  <si>
-    <t>Communication</t>
-  </si>
-  <si>
-    <t>From account creation</t>
-  </si>
-  <si>
-    <t>Google account &gt; Data &amp; privacy &gt; Download your data</t>
-  </si>
-  <si>
-    <t>.mbox or .zip</t>
-  </si>
-  <si>
     <t>Amazon</t>
   </si>
   <si>
@@ -110,10 +86,31 @@
     <t>.pdf</t>
   </si>
   <si>
-    <t>May include other Gmail services if selected.</t>
-  </si>
-  <si>
     <t>Puchase history may be split depending on delivery dates.</t>
+  </si>
+  <si>
+    <t>Google Chrome Browser</t>
+  </si>
+  <si>
+    <t>Autofill passwords</t>
+  </si>
+  <si>
+    <t>From account creation / any passwords that has been saved</t>
+  </si>
+  <si>
+    <t>.csv</t>
+  </si>
+  <si>
+    <t>Open browser &gt; Click the 3 dots to your top right corner &gt; Select "Passwords and autofill" &gt; Settings &gt; Click "download file" under "Export passwords"</t>
+  </si>
+  <si>
+    <t>This will only include passwords and login info that you opt in to save.</t>
+  </si>
+  <si>
+    <t>Log in &gt; Hover over "Account" to your top left corner &gt; Select "Statements and documents" &gt; Select "View" or "Download"</t>
+  </si>
+  <si>
+    <t>Statements</t>
   </si>
 </sst>
 </file>
@@ -491,16 +488,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CEEFA917-56F0-426C-A63C-C5FF40755B0A}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:G4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="18" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.6328125" style="1" customWidth="1"/>
     <col min="2" max="2" width="19.453125" style="2" customWidth="1"/>
-    <col min="3" max="3" width="19.26953125" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.26953125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="29" style="2" customWidth="1"/>
-    <col min="6" max="6" width="15.08984375" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="29.7265625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="20.1796875" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.26953125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="29.81640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.6328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="29.1796875" style="2" bestFit="1" customWidth="1"/>
     <col min="8" max="16384" width="8.7265625" style="1"/>
   </cols>
   <sheetData>
@@ -527,76 +527,77 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" ht="58" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>13</v>
-      </c>
     </row>
-    <row r="3" spans="1:7" ht="29" x14ac:dyDescent="0.35">
-      <c r="A3" s="1" t="s">
-        <v>14</v>
+    <row r="3" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
+      <c r="A3" s="2" t="s">
+        <v>17</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>16</v>
+        <v>18</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>19</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>25</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup scale="84" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>